<commit_message>
Add stop point functionality to video processing; enhance session control
</commit_message>
<xml_diff>
--- a/RecordingMeta.xlsx
+++ b/RecordingMeta.xlsx
@@ -1,110 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sachuriga/Desktop/code/HM_tracker_2025/HM_Tracker_2025/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47C1438C-B792-FD43-B50E-53B6ACCADF9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="680" windowWidth="28040" windowHeight="17320" xr2:uid="{76E3EA23-DBCA-4042-8441-5BD614C857C8}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="680" yWindow="680" windowWidth="28040" windowHeight="17320" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="181029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
-  <si>
-    <t>Rat_ID</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Repeat</t>
-  </si>
-  <si>
-    <t>Day</t>
-  </si>
-  <si>
-    <t>Session</t>
-  </si>
-  <si>
-    <t>Goal_Node</t>
-  </si>
-  <si>
-    <t>Prev_Goal_Node</t>
-  </si>
-  <si>
-    <t>Num_Trials</t>
-  </si>
-  <si>
-    <t>Start_Nodes</t>
-  </si>
-  <si>
-    <t>Special_Trials</t>
-  </si>
-  <si>
-    <t>Unnormal_Intervals</t>
-  </si>
-  <si>
-    <t>Start_Min</t>
-  </si>
-  <si>
-    <t>Start_Sec</t>
-  </si>
-  <si>
-    <t>Start_At_Trial_Num</t>
-  </si>
-  <si>
-    <t>1:0-5</t>
-  </si>
-  <si>
-    <t>3:10.3-12.4</t>
-  </si>
-  <si>
-    <t>Trial_Type</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -123,21 +46,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -457,127 +439,186 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FA2FE91-06CC-1B44-A119-622178D5BDE1}">
-  <dimension ref="A1:O6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Rat_ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Repeat</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Session</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Goal_Node</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Prev_Goal_Node</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Num_Trials</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Trial_Type</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Start_Nodes</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Special_Trials</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Unnormal_Intervals</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Start_Min</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Start_Sec</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Stop_Min</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Stop_Sec</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Start_At_Trial_Num</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B2" t="n">
+        <v>20210814</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>403</v>
+      </c>
+      <c r="G2" t="n">
+        <v>202</v>
+      </c>
+      <c r="H2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>102</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>1:0-5</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
+    </row>
+    <row r="3">
+      <c r="J3" t="n">
+        <v>304</v>
+      </c>
+      <c r="K3" t="n">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>16</v>
-      </c>
-      <c r="J1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" t="s">
-        <v>13</v>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>3:10.3-12.4</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>4</v>
-      </c>
-      <c r="B2">
-        <v>20210814</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>403</v>
-      </c>
-      <c r="G2">
-        <v>202</v>
-      </c>
-      <c r="H2">
-        <v>5</v>
-      </c>
-      <c r="I2">
-        <v>1</v>
-      </c>
-      <c r="J2">
+    <row r="4">
+      <c r="J4" t="n">
         <v>102</v>
       </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2" t="s">
-        <v>14</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2">
-        <v>0</v>
-      </c>
-      <c r="O2">
-        <v>1</v>
-      </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="J3">
-        <v>304</v>
-      </c>
-      <c r="K3">
-        <v>5</v>
-      </c>
-      <c r="L3" t="s">
-        <v>15</v>
+    <row r="5">
+      <c r="J5" t="n">
+        <v>405</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="J4">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="J5">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="J6">
+    <row r="6">
+      <c r="J6" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add termination time-locks for special trials; enforce end conditions based on scheduled times
</commit_message>
<xml_diff>
--- a/RecordingMeta.xlsx
+++ b/RecordingMeta.xlsx
@@ -444,9 +444,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
@@ -510,30 +512,35 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>Special_Trials_End</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>Unnormal_Intervals</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Start_Min</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Start_Sec</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Stop_Min</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Stop_Sec</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Start_At_Trial_Num</t>
         </is>
@@ -573,13 +580,10 @@
       <c r="K2" t="n">
         <v>1</v>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>1:0-5</t>
         </is>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
       </c>
       <c r="N2" t="n">
         <v>0</v>
@@ -591,6 +595,9 @@
         <v>0</v>
       </c>
       <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -601,7 +608,7 @@
       <c r="K3" t="n">
         <v>5</v>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>3:10.3-12.4</t>
         </is>

</xml_diff>